<commit_message>
Updated data dictionary and directory names
</commit_message>
<xml_diff>
--- a/Cleaned_Data/data_dictionary.xlsx
+++ b/Cleaned_Data/data_dictionary.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Stephanie/Documents/GitHub/mada-intestinal-parasites-prev/Cleaned_Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{32412EC0-E441-2646-B469-0D7C1F88FBD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8C8F995-29B4-A748-8197-CA838E8890FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4620" yWindow="3860" windowWidth="24520" windowHeight="14400" xr2:uid="{339A5614-6BD6-DC4B-8A79-A37F0C6EF25E}"/>
+    <workbookView xWindow="12060" yWindow="2740" windowWidth="17560" windowHeight="14400" activeTab="1" xr2:uid="{339A5614-6BD6-DC4B-8A79-A37F0C6EF25E}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="mah_dar_crs_fec_cleaned..." sheetId="1" r:id="rId1"/>
+    <sheet name="fec_key_bin_tp1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="68">
   <si>
     <t>Data dictionary for 'mah_dar_crs_fec_cleaned_avg_wide_public.csv'</t>
   </si>
@@ -53,15 +54,6 @@
     <t>ID</t>
   </si>
   <si>
-    <t>project_name</t>
-  </si>
-  <si>
-    <t>Project name. Either "mahery", "darwin", or "crs"</t>
-  </si>
-  <si>
-    <t>Individual ID composed of (project name)_(region)_(village)_(household)_(individual)_(timepoint)</t>
-  </si>
-  <si>
     <t>region</t>
   </si>
   <si>
@@ -300,6 +292,141 @@
   </si>
   <si>
     <t>Weight of the smear without liquid, in grams</t>
+  </si>
+  <si>
+    <t>Individual ID composed of (project name)_(region)_(village)_(household)_(individual)_(timepoint). Project name is either "mahery", "darwin", or "crs"</t>
+  </si>
+  <si>
+    <t>Data dictionary for 'fec_key_bin_tp1.csv'</t>
+  </si>
+  <si>
+    <t>Individual-level data with additional binary variables used for analysis. To prevent unstable estimates, data are subsetted to the first timepoint with data for each individual, for each parasite.</t>
+  </si>
+  <si>
+    <t>h_nana</t>
+  </si>
+  <si>
+    <t>s_mansoni</t>
+  </si>
+  <si>
+    <t>ascaris_bin</t>
+  </si>
+  <si>
+    <t>e_coli_bin</t>
+  </si>
+  <si>
+    <t>h_nana_bin</t>
+  </si>
+  <si>
+    <t>helms_bin</t>
+  </si>
+  <si>
+    <t>hook_bin</t>
+  </si>
+  <si>
+    <t>s_mansoni_bin</t>
+  </si>
+  <si>
+    <t>strongyloides_bin</t>
+  </si>
+  <si>
+    <t>trich_bin</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Binary 0/1 (no/yes) for presence of </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Ascaris lumbricoides</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Binary 0/1 (no/yes) for presence of </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Escherichia coli</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Binary 0/1 (no/yes) for presence of </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Hymenolepis nana</t>
+    </r>
+  </si>
+  <si>
+    <t>Binary 0/1 (no/yes) for presence of other helminths</t>
+  </si>
+  <si>
+    <t>Binary 0/1 (no/yes) for presence of hookworm</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Binary 0/1 (no/yes) for presence of </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Schistosoma mansoni</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Binary 0/1 (no/yes) for presence of </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Strongloides</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Binary 0/1 (no/yes) for presence of </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Trichuris trichiura</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -692,7 +819,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C498F2DD-8096-CE45-8C38-E03CC46F1351}">
-  <dimension ref="A1:B29"/>
+  <dimension ref="A1:B28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
@@ -727,7 +854,7 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>7</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -735,36 +862,36 @@
         <v>5</v>
       </c>
       <c r="B8" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B9" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
         <v>11</v>
-      </c>
-      <c r="B11" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B12" t="s">
         <v>14</v>
@@ -772,138 +899,383 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" t="s">
         <v>16</v>
-      </c>
-      <c r="B13" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>19</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B16" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B18" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B19" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B20" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B21" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B22" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B23" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B24" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B25" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B26" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B27" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
+        <v>31</v>
+      </c>
+      <c r="B28" t="s">
+        <v>45</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F49AEAD1-823F-8B4C-8808-8DD0D1A33915}">
+  <dimension ref="A1:B33"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="23.1640625" customWidth="1"/>
+    <col min="2" max="2" width="121.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>4</v>
+      </c>
+      <c r="B7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>6</v>
+      </c>
+      <c r="B9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>8</v>
+      </c>
+      <c r="B10" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>17</v>
+      </c>
+      <c r="B14" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B15" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>19</v>
+      </c>
+      <c r="B16" t="s">
         <v>33</v>
       </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>50</v>
+      </c>
+      <c r="B20" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>24</v>
+      </c>
+      <c r="B21" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>51</v>
+      </c>
+      <c r="B23" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>28</v>
+      </c>
+      <c r="B24" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>29</v>
+      </c>
+      <c r="B25" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>52</v>
+      </c>
+      <c r="B26" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>54</v>
+      </c>
       <c r="B28" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>34</v>
+        <v>55</v>
       </c>
       <c r="B29" t="s">
-        <v>48</v>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>56</v>
+      </c>
+      <c r="B30" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>57</v>
+      </c>
+      <c r="B31" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>58</v>
+      </c>
+      <c r="B32" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>59</v>
+      </c>
+      <c r="B33" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>

</xml_diff>